<commit_message>
Corrrection du bilan pour revenir à une approche plus proche du GRAFS original (pas de distinction organique naturel, pas de calcul de production de racines...).
</commit_message>
<xml_diff>
--- a/example/GRAFS_project_example_C_prospect.xlsx
+++ b/example/GRAFS_project_example_C_prospect.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\faustega\Documents\These\isterre-dynamic-modeling\grafs-e-project\grafs-e\example\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75222E22-61D0-48AE-93AB-1C89A3868944}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54431C93-6060-41A3-A6B4-9659D0A92F7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="16530" yWindow="-15870" windowWidth="25440" windowHeight="15270" activeTab="6" xr2:uid="{092E5AC7-17CB-4282-9989-CDCB089F75B9}"/>
+    <workbookView minimized="1" xWindow="2115" yWindow="-10335" windowWidth="14400" windowHeight="7275" xr2:uid="{092E5AC7-17CB-4282-9989-CDCB089F75B9}"/>
   </bookViews>
   <sheets>
     <sheet name="crops" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="109">
   <si>
     <t>Culture</t>
   </si>
@@ -267,9 +267,6 @@
     <t>Carbon Mechanisation Intensity (ktC/ha)</t>
   </si>
   <si>
-    <t>Surface Root Production (kgC/ha)</t>
-  </si>
-  <si>
     <t>Residue Humification Coefficient (%)</t>
   </si>
   <si>
@@ -367,6 +364,12 @@
   </si>
   <si>
     <t>Total Synthetic Fertilizer Use on crops (ktN)</t>
+  </si>
+  <si>
+    <t>Residue Nitrogen Content (%)</t>
+  </si>
+  <si>
+    <t>Weight synthetic distribution</t>
   </si>
 </sst>
 </file>
@@ -793,9 +796,9 @@
     <col min="9" max="9" width="25.54296875" customWidth="1"/>
     <col min="10" max="10" width="43" customWidth="1"/>
     <col min="11" max="11" width="25.54296875" customWidth="1"/>
-    <col min="12" max="13" width="37.81640625" customWidth="1"/>
-    <col min="14" max="14" width="32.1796875" customWidth="1"/>
-    <col min="15" max="15" width="28.81640625" customWidth="1"/>
+    <col min="12" max="12" width="29.08984375" customWidth="1"/>
+    <col min="13" max="14" width="37.81640625" customWidth="1"/>
+    <col min="15" max="15" width="32.1796875" customWidth="1"/>
     <col min="16" max="16" width="22.54296875" customWidth="1"/>
     <col min="17" max="17" width="32.81640625" customWidth="1"/>
   </cols>
@@ -823,22 +826,22 @@
         <v>50</v>
       </c>
       <c r="H1" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="I1" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="J1" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="K1" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="I1" s="5" t="s">
-        <v>88</v>
-      </c>
-      <c r="J1" s="5" t="s">
-        <v>106</v>
-      </c>
-      <c r="K1" s="5" t="s">
-        <v>86</v>
-      </c>
       <c r="L1" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="M1" s="5" t="s">
         <v>73</v>
-      </c>
-      <c r="M1" s="5" t="s">
-        <v>76</v>
       </c>
       <c r="N1" s="5" t="s">
         <v>75</v>
@@ -847,10 +850,10 @@
         <v>74</v>
       </c>
       <c r="P1" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="Q1" s="5" t="s">
         <v>104</v>
-      </c>
-      <c r="Q1" s="5" t="s">
-        <v>105</v>
       </c>
     </row>
     <row r="2" spans="1:17" ht="25" x14ac:dyDescent="0.35">
@@ -888,22 +891,22 @@
         <v>0</v>
       </c>
       <c r="L2" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="M2" s="3">
         <v>1E-4</v>
       </c>
-      <c r="M2" s="3">
+      <c r="N2" s="3">
         <v>40</v>
       </c>
-      <c r="N2" s="3">
+      <c r="O2" s="3">
         <v>22</v>
       </c>
-      <c r="O2" s="3">
-        <v>206</v>
-      </c>
       <c r="P2" s="3">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="Q2" s="3">
-        <v>180</v>
+        <v>246</v>
       </c>
     </row>
     <row r="3" spans="1:17" ht="25" x14ac:dyDescent="0.35">
@@ -941,22 +944,22 @@
         <v>0</v>
       </c>
       <c r="L3" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="M3" s="3">
         <v>1E-4</v>
       </c>
-      <c r="M3" s="3">
+      <c r="N3" s="3">
         <v>40</v>
       </c>
-      <c r="N3" s="3">
+      <c r="O3" s="3">
         <v>22</v>
       </c>
-      <c r="O3" s="3">
-        <v>136</v>
-      </c>
       <c r="P3" s="3">
-        <v>9</v>
+        <v>14.5</v>
       </c>
       <c r="Q3" s="3">
-        <v>140</v>
+        <v>213</v>
       </c>
     </row>
     <row r="4" spans="1:17" ht="25" x14ac:dyDescent="0.35">
@@ -994,22 +997,22 @@
         <v>0</v>
       </c>
       <c r="L4" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="M4" s="3">
         <v>1E-4</v>
       </c>
-      <c r="M4" s="3">
+      <c r="N4" s="3">
         <v>40</v>
       </c>
-      <c r="N4" s="3">
+      <c r="O4" s="3">
         <v>22</v>
       </c>
-      <c r="O4" s="3">
-        <v>500</v>
-      </c>
       <c r="P4" s="3">
-        <v>8</v>
+        <v>12.5</v>
       </c>
       <c r="Q4" s="3">
-        <v>80</v>
+        <v>216</v>
       </c>
     </row>
     <row r="5" spans="1:17" ht="25" x14ac:dyDescent="0.35">
@@ -1047,22 +1050,22 @@
         <v>0</v>
       </c>
       <c r="L5" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="M5" s="3">
         <v>1E-4</v>
       </c>
-      <c r="M5" s="3">
+      <c r="N5" s="3">
         <v>40</v>
       </c>
-      <c r="N5" s="3">
+      <c r="O5" s="3">
         <v>22</v>
       </c>
-      <c r="O5" s="3">
-        <v>300</v>
-      </c>
       <c r="P5" s="3">
-        <v>15</v>
+        <v>21.5</v>
       </c>
       <c r="Q5" s="3">
-        <v>180</v>
+        <v>293</v>
       </c>
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.35">
@@ -1100,22 +1103,22 @@
         <v>0</v>
       </c>
       <c r="L6" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="M6" s="3">
         <v>1E-4</v>
       </c>
-      <c r="M6" s="3">
+      <c r="N6" s="3">
         <v>40</v>
       </c>
-      <c r="N6" s="3">
+      <c r="O6" s="3">
         <v>22</v>
       </c>
-      <c r="O6" s="3">
-        <v>200</v>
-      </c>
       <c r="P6" s="3">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="Q6" s="3">
-        <v>120</v>
+        <v>562</v>
       </c>
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.35">
@@ -1153,22 +1156,22 @@
         <v>0</v>
       </c>
       <c r="L7" s="3">
+        <v>1.5</v>
+      </c>
+      <c r="M7" s="3">
         <v>1E-4</v>
       </c>
-      <c r="M7" s="3">
+      <c r="N7" s="3">
         <v>40</v>
       </c>
-      <c r="N7" s="3">
+      <c r="O7" s="3">
         <v>28</v>
       </c>
-      <c r="O7" s="3">
-        <v>50</v>
-      </c>
       <c r="P7" s="3">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Q7" s="3">
-        <v>50</v>
+        <v>6</v>
       </c>
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.35">
@@ -1179,7 +1182,7 @@
         <v>45</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D8" s="3">
         <v>0.77</v>
@@ -1206,16 +1209,16 @@
         <v>0</v>
       </c>
       <c r="L8" s="3">
+        <v>1</v>
+      </c>
+      <c r="M8" s="3">
         <v>5.0000000000000002E-5</v>
       </c>
-      <c r="M8" s="3">
+      <c r="N8" s="3">
         <v>40</v>
       </c>
-      <c r="N8" s="3">
+      <c r="O8" s="3">
         <v>25</v>
-      </c>
-      <c r="O8" s="3">
-        <v>600</v>
       </c>
       <c r="P8" s="3">
         <v>8</v>
@@ -1226,13 +1229,13 @@
     </row>
     <row r="9" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
+        <v>82</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="C9" s="2" t="s">
         <v>83</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>84</v>
       </c>
       <c r="D9" s="3">
         <v>0</v>
@@ -1259,7 +1262,7 @@
         <v>0</v>
       </c>
       <c r="L9" s="3">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="M9" s="3">
         <v>0</v>
@@ -1271,10 +1274,10 @@
         <v>0</v>
       </c>
       <c r="P9" s="3">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="Q9" s="3">
-        <v>250</v>
+        <v>150</v>
       </c>
     </row>
   </sheetData>
@@ -1405,33 +1408,33 @@
   <sheetData>
     <row r="1" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="B1" s="5" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="5" t="s">
-        <v>91</v>
-      </c>
       <c r="C1" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D1" s="5" t="s">
         <v>10</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
+        <v>91</v>
+      </c>
+      <c r="B2" t="s">
         <v>92</v>
-      </c>
-      <c r="B2" t="s">
-        <v>93</v>
       </c>
       <c r="C2">
         <v>1000</v>
       </c>
       <c r="D2" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="E2">
         <v>5</v>
@@ -1439,16 +1442,16 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
+        <v>93</v>
+      </c>
+      <c r="B3" t="s">
         <v>94</v>
-      </c>
-      <c r="B3" t="s">
-        <v>95</v>
       </c>
       <c r="C3">
         <v>100</v>
       </c>
       <c r="D3" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E3">
         <v>10</v>
@@ -1503,7 +1506,7 @@
         <v>68</v>
       </c>
       <c r="J1" s="5" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="K1" s="5" t="s">
         <v>29</v>
@@ -1707,13 +1710,13 @@
         <v>52</v>
       </c>
       <c r="G1" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="H1" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="H1" s="5" t="s">
-        <v>78</v>
-      </c>
       <c r="I1" s="5" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.35">
@@ -1901,7 +1904,7 @@
         <v>19</v>
       </c>
       <c r="D8" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E8">
         <v>2.0499999999999998</v>
@@ -2037,16 +2040,16 @@
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
+        <v>81</v>
+      </c>
+      <c r="B13" t="s">
         <v>82</v>
-      </c>
-      <c r="B13" t="s">
-        <v>83</v>
       </c>
       <c r="C13" t="s">
         <v>19</v>
       </c>
       <c r="D13" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E13">
         <v>2</v>
@@ -2072,7 +2075,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{986D1BE3-7A15-4223-93AE-9AB753B07534}">
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="50.81640625" customWidth="1"/>
@@ -2128,7 +2131,7 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B7">
         <v>10</v>
@@ -2136,7 +2139,7 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B8">
         <v>0.1</v>
@@ -2144,7 +2147,7 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B9">
         <v>1</v>
@@ -2152,7 +2155,7 @@
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B10">
         <v>10</v>
@@ -2160,7 +2163,7 @@
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B11">
         <v>1</v>
@@ -2168,7 +2171,7 @@
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B12">
         <v>1</v>
@@ -2176,7 +2179,7 @@
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B13">
         <v>1</v>
@@ -2184,10 +2187,18 @@
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B14">
-        <v>1000</v>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>106</v>
+      </c>
+      <c r="B15">
+        <v>2000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>